<commit_message>
Actualizar componentes y datasheets
</commit_message>
<xml_diff>
--- a/Tablas/BOM_CubeSat_1U_OBC_Comms.xlsx
+++ b/Tablas/BOM_CubeSat_1U_OBC_Comms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juan_diaz/Documents/UdeA/Electronica/Semestre_8/Diseno/Proyecto_Diseno_Productos/Tablas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Base_User\UdeA\Electronica\Semestre_8\Diseño\Lab4\Proyecto_Diseno_Productos\Tablas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9344A7A7-7057-A049-93EF-85C25D6C9588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A04B50-CAEC-4365-B4DC-3C525A35E097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lista de Componentes" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="120">
   <si>
     <t>Categoría</t>
   </si>
@@ -119,18 +119,9 @@
     <t>Reloj / Oscilador</t>
   </si>
   <si>
-    <t>Rakon</t>
-  </si>
-  <si>
-    <t>RPT7050A</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
-    <t>Sin verificar. Opcional, basta un industrial estándar.</t>
-  </si>
-  <si>
     <t>Supervisor / Watchdog</t>
   </si>
   <si>
@@ -191,9 +182,6 @@
     <t>Qorvo</t>
   </si>
   <si>
-    <t>TQP3M9018</t>
-  </si>
-  <si>
     <t>5 V</t>
   </si>
   <si>
@@ -257,9 +245,6 @@
     <t>Filtro de TX</t>
   </si>
   <si>
-    <t>2450BP15H0100</t>
-  </si>
-  <si>
     <t>Pérdida 1.8 dB. Soporta 2 W.</t>
   </si>
   <si>
@@ -284,21 +269,12 @@
     <t>Regulador Switching (Buck)</t>
   </si>
   <si>
-    <t>TPS62130A-Q1</t>
-  </si>
-  <si>
     <t>Varios (1.2V, 1.35V, 1.8V, 3.3V)</t>
   </si>
   <si>
     <t>LDO de Ultra Bajo Ruido</t>
   </si>
   <si>
-    <t>LT3042 / LT3045</t>
-  </si>
-  <si>
-    <t>1.3 V</t>
-  </si>
-  <si>
     <t>Sin verificar. Esencial para limpiar el AD9364.</t>
   </si>
   <si>
@@ -332,9 +308,6 @@
     <t>Samtec</t>
   </si>
   <si>
-    <t>FTSH-105-01-L-DV</t>
-  </si>
-  <si>
     <t>Conector Bus CubeSat (PC/104)</t>
   </si>
   <si>
@@ -347,9 +320,6 @@
     <t>Conectores de Antena</t>
   </si>
   <si>
-    <t>SMP o MMCX</t>
-  </si>
-  <si>
     <t>Materiales PCB (Stackup)</t>
   </si>
   <si>
@@ -365,7 +335,64 @@
     <t>Harwin</t>
   </si>
   <si>
-    <t>TCXO de 40 MHz (RST2016A)</t>
+    <t>Aker</t>
+  </si>
+  <si>
+    <t>S3A33025</t>
+  </si>
+  <si>
+    <t>3,3 V</t>
+  </si>
+  <si>
+    <t>Reloj Oscilador 50 Mhz</t>
+  </si>
+  <si>
+    <t>PSA4-5043</t>
+  </si>
+  <si>
+    <t>3/5 V</t>
+  </si>
+  <si>
+    <t>S733025T</t>
+  </si>
+  <si>
+    <t>3.3V</t>
+  </si>
+  <si>
+    <t>Oscilador 40 MHz</t>
+  </si>
+  <si>
+    <t>DEA202450BT</t>
+  </si>
+  <si>
+    <t>TDK</t>
+  </si>
+  <si>
+    <t>TPS62903</t>
+  </si>
+  <si>
+    <t>LT3045</t>
+  </si>
+  <si>
+    <t>Regulador Ajustable 0-15V</t>
+  </si>
+  <si>
+    <t>HTST10501 -LDVDA</t>
+  </si>
+  <si>
+    <t>10 pines</t>
+  </si>
+  <si>
+    <t>52 Pines</t>
+  </si>
+  <si>
+    <t>18S142-40ML5</t>
+  </si>
+  <si>
+    <t>Rosenberger</t>
+  </si>
+  <si>
+    <t>Conector SMP</t>
   </si>
 </sst>
 </file>
@@ -740,7 +767,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -749,7 +776,7 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -769,7 +796,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -789,7 +816,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -809,7 +836,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -829,7 +856,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -849,7 +876,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -857,473 +884,473 @@
         <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="E8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="D21" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="2" t="s">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B23" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="D28" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>21</v>

</xml_diff>